<commit_message>
output, and debugging for multiple vehicles/trips when not needed
</commit_message>
<xml_diff>
--- a/notebooks/outputs/prm_v2/monthly_summary/monthly_summary.xlsx
+++ b/notebooks/outputs/prm_v2/monthly_summary/monthly_summary.xlsx
@@ -13,10 +13,80 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="19">
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>mode</t>
+  </si>
+  <si>
+    <t>arrival_sla_pct</t>
+  </si>
+  <si>
+    <t>peak_amb</t>
+  </si>
+  <si>
+    <t>peak_mini</t>
+  </si>
+  <si>
+    <t>peak_staff</t>
+  </si>
+  <si>
+    <t>fleet_expansion_required</t>
+  </si>
+  <si>
+    <t>current_fleet_sufficient</t>
+  </si>
+  <si>
+    <t>recommended_scenario</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>P100</t>
+  </si>
+  <si>
+    <t>P90</t>
+  </si>
+  <si>
+    <t>CURRENT_FLEET_OK</t>
+  </si>
+  <si>
+    <t>p90_future_plus_1</t>
+  </si>
+  <si>
+    <t>p100_future_plus_1</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -32,7 +102,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -40,12 +110,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -340,9 +428,329 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2">
+        <v>100</v>
+      </c>
+      <c r="D2">
+        <v>11</v>
+      </c>
+      <c r="E2">
+        <v>3</v>
+      </c>
+      <c r="F2">
+        <v>43</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3">
+        <v>100</v>
+      </c>
+      <c r="D3">
+        <v>12</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3">
+        <v>41</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4">
+        <v>100</v>
+      </c>
+      <c r="D4">
+        <v>11</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4">
+        <v>55</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5">
+        <v>100</v>
+      </c>
+      <c r="D5">
+        <v>12</v>
+      </c>
+      <c r="E5">
+        <v>3</v>
+      </c>
+      <c r="F5">
+        <v>41</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6">
+        <v>99.84981515711645</v>
+      </c>
+      <c r="D6">
+        <v>9</v>
+      </c>
+      <c r="E6">
+        <v>3</v>
+      </c>
+      <c r="F6">
+        <v>37</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7">
+        <v>100</v>
+      </c>
+      <c r="D7">
+        <v>8</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>34</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8">
+        <v>100</v>
+      </c>
+      <c r="D8">
+        <v>10</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+      <c r="F8">
+        <v>54</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9">
+        <v>100</v>
+      </c>
+      <c r="D9">
+        <v>9</v>
+      </c>
+      <c r="E9">
+        <v>3</v>
+      </c>
+      <c r="F9">
+        <v>42</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10">
+        <v>100</v>
+      </c>
+      <c r="D10">
+        <v>11</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10">
+        <v>59</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11">
+        <v>100</v>
+      </c>
+      <c r="D11">
+        <v>9</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11">
+        <v>45</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>